<commit_message>
New part number added
</commit_message>
<xml_diff>
--- a/hardware/pcb/LED_board_iorodeo/assembly/BOM_JLCPCB_radial_16mA.xlsx
+++ b/hardware/pcb/LED_board_iorodeo/assembly/BOM_JLCPCB_radial_16mA.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
   <si>
     <t>Comment</t>
   </si>
@@ -197,12 +197,21 @@
   <si>
     <t>PJSEMI</t>
   </si>
+  <si>
+    <t>LMV321</t>
+  </si>
+  <si>
+    <t>C7972</t>
+  </si>
+  <si>
+    <t>vor 11 Stunden</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -237,6 +246,12 @@
       <color rgb="FF000000"/>
       <name val="宋体"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F2328"/>
+      <name val="Segoe UI"/>
+      <family val="18"/>
     </font>
   </fonts>
   <fills count="4">
@@ -288,7 +303,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -312,6 +327,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -715,7 +733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AMJ11"/>
+  <dimension ref="A1:AMJ12"/>
   <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="13.5" x14ac:dyDescent="0.1"/>
   <cols>
     <col min="1" max="1" width="52.08984375" style="1" customWidth="1"/>
@@ -916,6 +934,23 @@
         <v>41</v>
       </c>
     </row>
+    <row r="12" spans="1:6" ht="16.5" x14ac:dyDescent="0.1">
+      <c r="A12" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="1">
+        <v>1</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>